<commit_message>
release: freeze reproducible 2026.07.27.1
</commit_message>
<xml_diff>
--- a/virus_detect.xlsx
+++ b/virus_detect.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wuhhh/Desktop/徐老师/代码/metagenomic/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBAF5745-1184-6642-9D3B-08282F4167E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E161383-D207-F44A-8921-04CA05FBAE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16280" xr2:uid="{8AF6CC31-C9CD-6745-986E-91C6053BA279}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="215">
   <si>
     <t>一级分类</t>
   </si>
@@ -1066,6 +1066,7 @@
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
     <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1586,8 +1587,8 @@
       <c r="H19" t="s">
         <v>79</v>
       </c>
-      <c r="I19" s="1" t="s">
-        <v>211</v>
+      <c r="I19" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1615,8 +1616,8 @@
       <c r="H20" t="s">
         <v>79</v>
       </c>
-      <c r="I20" s="1" t="s">
-        <v>211</v>
+      <c r="I20" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1644,8 +1645,8 @@
       <c r="H21" t="s">
         <v>113</v>
       </c>
-      <c r="I21" s="1" t="s">
-        <v>211</v>
+      <c r="I21" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1673,8 +1674,8 @@
       <c r="H22" t="s">
         <v>113</v>
       </c>
-      <c r="I22" s="1" t="s">
-        <v>211</v>
+      <c r="I22" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1731,8 +1732,8 @@
       <c r="H25" t="s">
         <v>128</v>
       </c>
-      <c r="I25" s="1" t="s">
-        <v>212</v>
+      <c r="I25" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1948,6 +1949,9 @@
       <c r="H34" t="s">
         <v>79</v>
       </c>
+      <c r="I34" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
@@ -1973,6 +1977,9 @@
       </c>
       <c r="H35" t="s">
         <v>169</v>
+      </c>
+      <c r="I35" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="36" spans="1:9">

</xml_diff>